<commit_message>
Add two performance charts to KPI Dashboard
- Chart 1 (26x15cm): Stacked column (Umsatz per employee per month) with
  cumulative trend line on secondary axis – shows team total as bar height
  and overall growth trajectory as smooth anthracite line
- Chart 2 (22x12cm): Clustered column (Abschluesse per employee per month)
- Helper table at row 110-123 with SUMPRODUCT formulas for monthly aggregation
  (Umsatz, Abschluesse, neue Leads, kumulierter Umsatz) per employee
- Fitshop colors per employee: Daniel=rot, Jonas=blau, Angie=gruen, Norbert=orange

https://claude.ai/code/session_01WiRUeJ8tQNpk2kLkUtpvQn
</commit_message>
<xml_diff>
--- a/fitshop-sop/Fitshop_Tracking_2026.xlsx
+++ b/fitshop-sop/Fitshop_Tracking_2026.xlsx
@@ -23,7 +23,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="#,##0 &quot;EUR&quot;"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -82,6 +82,19 @@
       <name val="Calibri"/>
       <color rgb="00000000"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <i val="1"/>
+      <color rgb="00AAAAAA"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="8"/>
     </font>
   </fonts>
   <fills count="12">
@@ -206,7 +219,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -278,6 +291,16 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -558,6 +581,549 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="10"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Umsatz-Entwicklung 2026 nach Mitarbeiter (EUR)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="stacked"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'KPI Dashboard'!C111</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:solidFill>
+              <a:srgbClr val="E31E24"/>
+            </a:solidFill>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="E31E24"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'KPI Dashboard'!$A$112:$A$123</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'KPI Dashboard'!$C$112:$C$123</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'KPI Dashboard'!D111</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:solidFill>
+              <a:srgbClr val="1565C0"/>
+            </a:solidFill>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="1565C0"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'KPI Dashboard'!$A$112:$A$123</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'KPI Dashboard'!$D$112:$D$123</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="2"/>
+          <order val="2"/>
+          <tx>
+            <strRef>
+              <f>'KPI Dashboard'!E111</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:solidFill>
+              <a:srgbClr val="2E7D32"/>
+            </a:solidFill>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="2E7D32"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'KPI Dashboard'!$A$112:$A$123</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'KPI Dashboard'!$E$112:$E$123</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="3"/>
+          <order val="3"/>
+          <tx>
+            <strRef>
+              <f>'KPI Dashboard'!F111</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:solidFill>
+              <a:srgbClr val="E65100"/>
+            </a:solidFill>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="E65100"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'KPI Dashboard'!$A$112:$A$123</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'KPI Dashboard'!$F$112:$F$123</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <overlap val="100"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="4"/>
+          <order val="4"/>
+          <tx>
+            <strRef>
+              <f>'KPI Dashboard'!M111</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln w="31750">
+              <a:solidFill>
+                <a:srgbClr val="2D2D2D"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="circle"/>
+            <size val="6"/>
+            <spPr>
+              <a:solidFill>
+                <a:srgbClr val="2D2D2D"/>
+              </a:solidFill>
+              <a:ln>
+                <a:solidFill>
+                  <a:srgbClr val="2D2D2D"/>
+                </a:solidFill>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'KPI Dashboard'!$A$112:$A$123</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'KPI Dashboard'!$M$112:$M$123</f>
+            </numRef>
+          </val>
+          <smooth val="1"/>
+        </ser>
+        <axId val="10"/>
+        <axId val="200"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Monat</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>EUR (monatlich)</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+      <valAx>
+        <axId val="200"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Kumuliert (EUR)</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+        <crosses val="max"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="10"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Abschlüsse pro Monat nach Mitarbeiter</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'KPI Dashboard'!H111</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:solidFill>
+              <a:srgbClr val="E31E24"/>
+            </a:solidFill>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="E31E24"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'KPI Dashboard'!$A$112:$A$123</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'KPI Dashboard'!$H$112:$H$123</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'KPI Dashboard'!I111</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:solidFill>
+              <a:srgbClr val="1565C0"/>
+            </a:solidFill>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="1565C0"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'KPI Dashboard'!$A$112:$A$123</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'KPI Dashboard'!$I$112:$I$123</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="2"/>
+          <order val="2"/>
+          <tx>
+            <strRef>
+              <f>'KPI Dashboard'!J111</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:solidFill>
+              <a:srgbClr val="2E7D32"/>
+            </a:solidFill>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="2E7D32"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'KPI Dashboard'!$A$112:$A$123</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'KPI Dashboard'!$J$112:$J$123</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="3"/>
+          <order val="3"/>
+          <tx>
+            <strRef>
+              <f>'KPI Dashboard'!K111</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:solidFill>
+              <a:srgbClr val="E65100"/>
+            </a:solidFill>
+            <a:ln>
+              <a:solidFill>
+                <a:srgbClr val="E65100"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'KPI Dashboard'!$A$112:$A$123</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'KPI Dashboard'!$K$112:$K$123</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Monat</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Anzahl Abschlüsse</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>25</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="9360000" cy="5400000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>48</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="7920000" cy="4320000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="2" name="Chart 2"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -6088,7 +6654,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:M123"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -6097,6 +6663,13 @@
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="13" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="38" customHeight="1">
@@ -6500,12 +7073,763 @@
       <c r="E21" s="23" t="n"/>
       <c r="F21" s="23" t="n"/>
     </row>
+    <row r="24" ht="22" customHeight="1">
+      <c r="A24" s="20" t="inlineStr">
+        <is>
+          <t>LEISTUNGSENTWICKLUNG 2026 – GRAFIKEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="15" customHeight="1">
+      <c r="A25" s="10" t="inlineStr">
+        <is>
+          <t>Daten werden automatisch aus dem Lead-Tracking gezogen. Ansicht aktualisieren: Strg+Alt+F9</t>
+        </is>
+      </c>
+    </row>
+    <row r="110" ht="16" customHeight="1">
+      <c r="A110" s="27" t="inlineStr">
+        <is>
+          <t>CHART-DATEN (automatisch berechnet – nicht bearbeiten)</t>
+        </is>
+      </c>
+    </row>
+    <row r="111" ht="20" customHeight="1">
+      <c r="A111" s="28" t="inlineStr">
+        <is>
+          <t>Monat</t>
+        </is>
+      </c>
+      <c r="B111" s="28" t="inlineStr">
+        <is>
+          <t>Umsatz Ges.</t>
+        </is>
+      </c>
+      <c r="C111" s="28" t="inlineStr">
+        <is>
+          <t>Daniel EUR</t>
+        </is>
+      </c>
+      <c r="D111" s="28" t="inlineStr">
+        <is>
+          <t>Jonas EUR</t>
+        </is>
+      </c>
+      <c r="E111" s="28" t="inlineStr">
+        <is>
+          <t>Angie EUR</t>
+        </is>
+      </c>
+      <c r="F111" s="28" t="inlineStr">
+        <is>
+          <t>Norbert EUR</t>
+        </is>
+      </c>
+      <c r="G111" s="28" t="inlineStr">
+        <is>
+          <t>Abschl. Ges.</t>
+        </is>
+      </c>
+      <c r="H111" s="28" t="inlineStr">
+        <is>
+          <t>Daniel #</t>
+        </is>
+      </c>
+      <c r="I111" s="28" t="inlineStr">
+        <is>
+          <t>Jonas #</t>
+        </is>
+      </c>
+      <c r="J111" s="28" t="inlineStr">
+        <is>
+          <t>Angie #</t>
+        </is>
+      </c>
+      <c r="K111" s="28" t="inlineStr">
+        <is>
+          <t>Norbert #</t>
+        </is>
+      </c>
+      <c r="L111" s="28" t="inlineStr">
+        <is>
+          <t>Neue Leads</t>
+        </is>
+      </c>
+      <c r="M111" s="28" t="inlineStr">
+        <is>
+          <t>Kum. Umsatz</t>
+        </is>
+      </c>
+    </row>
+    <row r="112" ht="18" customHeight="1">
+      <c r="A112" s="29" t="inlineStr">
+        <is>
+          <t>Januar</t>
+        </is>
+      </c>
+      <c r="B112" s="30">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=1)*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
+        <v/>
+      </c>
+      <c r="C112" s="30">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=1)*('Lead-Tracking 2026'!$C$4:$C$2000="Daniel")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
+        <v/>
+      </c>
+      <c r="D112" s="30">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=1)*('Lead-Tracking 2026'!$C$4:$C$2000="Jonas")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
+        <v/>
+      </c>
+      <c r="E112" s="30">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=1)*('Lead-Tracking 2026'!$C$4:$C$2000="Angie")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
+        <v/>
+      </c>
+      <c r="F112" s="30">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=1)*('Lead-Tracking 2026'!$C$4:$C$2000="Norbert")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
+        <v/>
+      </c>
+      <c r="G112" s="30">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=1)*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
+        <v/>
+      </c>
+      <c r="H112" s="30">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=1)*('Lead-Tracking 2026'!$C$4:$C$2000="Daniel")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
+        <v/>
+      </c>
+      <c r="I112" s="30">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=1)*('Lead-Tracking 2026'!$C$4:$C$2000="Jonas")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
+        <v/>
+      </c>
+      <c r="J112" s="30">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=1)*('Lead-Tracking 2026'!$C$4:$C$2000="Angie")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
+        <v/>
+      </c>
+      <c r="K112" s="30">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=1)*('Lead-Tracking 2026'!$C$4:$C$2000="Norbert")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
+        <v/>
+      </c>
+      <c r="L112" s="30">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=1)*('Lead-Tracking 2026'!$A$4:$A$2000&lt;&gt;""))</f>
+        <v/>
+      </c>
+      <c r="M112" s="30">
+        <f>B112</f>
+        <v/>
+      </c>
+    </row>
+    <row r="113" ht="18" customHeight="1">
+      <c r="A113" s="31" t="inlineStr">
+        <is>
+          <t>Februar</t>
+        </is>
+      </c>
+      <c r="B113" s="32">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=2)*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
+        <v/>
+      </c>
+      <c r="C113" s="32">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=2)*('Lead-Tracking 2026'!$C$4:$C$2000="Daniel")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
+        <v/>
+      </c>
+      <c r="D113" s="32">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=2)*('Lead-Tracking 2026'!$C$4:$C$2000="Jonas")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
+        <v/>
+      </c>
+      <c r="E113" s="32">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=2)*('Lead-Tracking 2026'!$C$4:$C$2000="Angie")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
+        <v/>
+      </c>
+      <c r="F113" s="32">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=2)*('Lead-Tracking 2026'!$C$4:$C$2000="Norbert")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
+        <v/>
+      </c>
+      <c r="G113" s="32">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=2)*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
+        <v/>
+      </c>
+      <c r="H113" s="32">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=2)*('Lead-Tracking 2026'!$C$4:$C$2000="Daniel")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
+        <v/>
+      </c>
+      <c r="I113" s="32">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=2)*('Lead-Tracking 2026'!$C$4:$C$2000="Jonas")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
+        <v/>
+      </c>
+      <c r="J113" s="32">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=2)*('Lead-Tracking 2026'!$C$4:$C$2000="Angie")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
+        <v/>
+      </c>
+      <c r="K113" s="32">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=2)*('Lead-Tracking 2026'!$C$4:$C$2000="Norbert")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
+        <v/>
+      </c>
+      <c r="L113" s="32">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=2)*('Lead-Tracking 2026'!$A$4:$A$2000&lt;&gt;""))</f>
+        <v/>
+      </c>
+      <c r="M113" s="32">
+        <f>M112+B113</f>
+        <v/>
+      </c>
+    </row>
+    <row r="114" ht="18" customHeight="1">
+      <c r="A114" s="29" t="inlineStr">
+        <is>
+          <t>März</t>
+        </is>
+      </c>
+      <c r="B114" s="30">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=3)*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
+        <v/>
+      </c>
+      <c r="C114" s="30">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=3)*('Lead-Tracking 2026'!$C$4:$C$2000="Daniel")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
+        <v/>
+      </c>
+      <c r="D114" s="30">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=3)*('Lead-Tracking 2026'!$C$4:$C$2000="Jonas")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
+        <v/>
+      </c>
+      <c r="E114" s="30">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=3)*('Lead-Tracking 2026'!$C$4:$C$2000="Angie")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
+        <v/>
+      </c>
+      <c r="F114" s="30">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=3)*('Lead-Tracking 2026'!$C$4:$C$2000="Norbert")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
+        <v/>
+      </c>
+      <c r="G114" s="30">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=3)*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
+        <v/>
+      </c>
+      <c r="H114" s="30">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=3)*('Lead-Tracking 2026'!$C$4:$C$2000="Daniel")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
+        <v/>
+      </c>
+      <c r="I114" s="30">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=3)*('Lead-Tracking 2026'!$C$4:$C$2000="Jonas")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
+        <v/>
+      </c>
+      <c r="J114" s="30">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=3)*('Lead-Tracking 2026'!$C$4:$C$2000="Angie")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
+        <v/>
+      </c>
+      <c r="K114" s="30">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=3)*('Lead-Tracking 2026'!$C$4:$C$2000="Norbert")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
+        <v/>
+      </c>
+      <c r="L114" s="30">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=3)*('Lead-Tracking 2026'!$A$4:$A$2000&lt;&gt;""))</f>
+        <v/>
+      </c>
+      <c r="M114" s="30">
+        <f>M113+B114</f>
+        <v/>
+      </c>
+    </row>
+    <row r="115" ht="18" customHeight="1">
+      <c r="A115" s="31" t="inlineStr">
+        <is>
+          <t>April</t>
+        </is>
+      </c>
+      <c r="B115" s="32">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=4)*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
+        <v/>
+      </c>
+      <c r="C115" s="32">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=4)*('Lead-Tracking 2026'!$C$4:$C$2000="Daniel")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
+        <v/>
+      </c>
+      <c r="D115" s="32">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=4)*('Lead-Tracking 2026'!$C$4:$C$2000="Jonas")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
+        <v/>
+      </c>
+      <c r="E115" s="32">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=4)*('Lead-Tracking 2026'!$C$4:$C$2000="Angie")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
+        <v/>
+      </c>
+      <c r="F115" s="32">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=4)*('Lead-Tracking 2026'!$C$4:$C$2000="Norbert")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
+        <v/>
+      </c>
+      <c r="G115" s="32">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=4)*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
+        <v/>
+      </c>
+      <c r="H115" s="32">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=4)*('Lead-Tracking 2026'!$C$4:$C$2000="Daniel")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
+        <v/>
+      </c>
+      <c r="I115" s="32">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=4)*('Lead-Tracking 2026'!$C$4:$C$2000="Jonas")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
+        <v/>
+      </c>
+      <c r="J115" s="32">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=4)*('Lead-Tracking 2026'!$C$4:$C$2000="Angie")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
+        <v/>
+      </c>
+      <c r="K115" s="32">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=4)*('Lead-Tracking 2026'!$C$4:$C$2000="Norbert")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
+        <v/>
+      </c>
+      <c r="L115" s="32">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=4)*('Lead-Tracking 2026'!$A$4:$A$2000&lt;&gt;""))</f>
+        <v/>
+      </c>
+      <c r="M115" s="32">
+        <f>M114+B115</f>
+        <v/>
+      </c>
+    </row>
+    <row r="116" ht="18" customHeight="1">
+      <c r="A116" s="29" t="inlineStr">
+        <is>
+          <t>Mai</t>
+        </is>
+      </c>
+      <c r="B116" s="30">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=5)*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
+        <v/>
+      </c>
+      <c r="C116" s="30">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=5)*('Lead-Tracking 2026'!$C$4:$C$2000="Daniel")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
+        <v/>
+      </c>
+      <c r="D116" s="30">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=5)*('Lead-Tracking 2026'!$C$4:$C$2000="Jonas")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
+        <v/>
+      </c>
+      <c r="E116" s="30">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=5)*('Lead-Tracking 2026'!$C$4:$C$2000="Angie")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
+        <v/>
+      </c>
+      <c r="F116" s="30">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=5)*('Lead-Tracking 2026'!$C$4:$C$2000="Norbert")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
+        <v/>
+      </c>
+      <c r="G116" s="30">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=5)*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
+        <v/>
+      </c>
+      <c r="H116" s="30">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=5)*('Lead-Tracking 2026'!$C$4:$C$2000="Daniel")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
+        <v/>
+      </c>
+      <c r="I116" s="30">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=5)*('Lead-Tracking 2026'!$C$4:$C$2000="Jonas")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
+        <v/>
+      </c>
+      <c r="J116" s="30">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=5)*('Lead-Tracking 2026'!$C$4:$C$2000="Angie")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
+        <v/>
+      </c>
+      <c r="K116" s="30">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=5)*('Lead-Tracking 2026'!$C$4:$C$2000="Norbert")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
+        <v/>
+      </c>
+      <c r="L116" s="30">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=5)*('Lead-Tracking 2026'!$A$4:$A$2000&lt;&gt;""))</f>
+        <v/>
+      </c>
+      <c r="M116" s="30">
+        <f>M115+B116</f>
+        <v/>
+      </c>
+    </row>
+    <row r="117" ht="18" customHeight="1">
+      <c r="A117" s="31" t="inlineStr">
+        <is>
+          <t>Juni</t>
+        </is>
+      </c>
+      <c r="B117" s="32">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=6)*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
+        <v/>
+      </c>
+      <c r="C117" s="32">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=6)*('Lead-Tracking 2026'!$C$4:$C$2000="Daniel")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
+        <v/>
+      </c>
+      <c r="D117" s="32">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=6)*('Lead-Tracking 2026'!$C$4:$C$2000="Jonas")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
+        <v/>
+      </c>
+      <c r="E117" s="32">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=6)*('Lead-Tracking 2026'!$C$4:$C$2000="Angie")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
+        <v/>
+      </c>
+      <c r="F117" s="32">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=6)*('Lead-Tracking 2026'!$C$4:$C$2000="Norbert")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
+        <v/>
+      </c>
+      <c r="G117" s="32">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=6)*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
+        <v/>
+      </c>
+      <c r="H117" s="32">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=6)*('Lead-Tracking 2026'!$C$4:$C$2000="Daniel")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
+        <v/>
+      </c>
+      <c r="I117" s="32">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=6)*('Lead-Tracking 2026'!$C$4:$C$2000="Jonas")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
+        <v/>
+      </c>
+      <c r="J117" s="32">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=6)*('Lead-Tracking 2026'!$C$4:$C$2000="Angie")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
+        <v/>
+      </c>
+      <c r="K117" s="32">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=6)*('Lead-Tracking 2026'!$C$4:$C$2000="Norbert")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
+        <v/>
+      </c>
+      <c r="L117" s="32">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=6)*('Lead-Tracking 2026'!$A$4:$A$2000&lt;&gt;""))</f>
+        <v/>
+      </c>
+      <c r="M117" s="32">
+        <f>M116+B117</f>
+        <v/>
+      </c>
+    </row>
+    <row r="118" ht="18" customHeight="1">
+      <c r="A118" s="29" t="inlineStr">
+        <is>
+          <t>Juli</t>
+        </is>
+      </c>
+      <c r="B118" s="30">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=7)*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
+        <v/>
+      </c>
+      <c r="C118" s="30">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=7)*('Lead-Tracking 2026'!$C$4:$C$2000="Daniel")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
+        <v/>
+      </c>
+      <c r="D118" s="30">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=7)*('Lead-Tracking 2026'!$C$4:$C$2000="Jonas")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
+        <v/>
+      </c>
+      <c r="E118" s="30">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=7)*('Lead-Tracking 2026'!$C$4:$C$2000="Angie")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
+        <v/>
+      </c>
+      <c r="F118" s="30">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=7)*('Lead-Tracking 2026'!$C$4:$C$2000="Norbert")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
+        <v/>
+      </c>
+      <c r="G118" s="30">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=7)*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
+        <v/>
+      </c>
+      <c r="H118" s="30">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=7)*('Lead-Tracking 2026'!$C$4:$C$2000="Daniel")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
+        <v/>
+      </c>
+      <c r="I118" s="30">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=7)*('Lead-Tracking 2026'!$C$4:$C$2000="Jonas")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
+        <v/>
+      </c>
+      <c r="J118" s="30">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=7)*('Lead-Tracking 2026'!$C$4:$C$2000="Angie")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
+        <v/>
+      </c>
+      <c r="K118" s="30">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=7)*('Lead-Tracking 2026'!$C$4:$C$2000="Norbert")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
+        <v/>
+      </c>
+      <c r="L118" s="30">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=7)*('Lead-Tracking 2026'!$A$4:$A$2000&lt;&gt;""))</f>
+        <v/>
+      </c>
+      <c r="M118" s="30">
+        <f>M117+B118</f>
+        <v/>
+      </c>
+    </row>
+    <row r="119" ht="18" customHeight="1">
+      <c r="A119" s="31" t="inlineStr">
+        <is>
+          <t>August</t>
+        </is>
+      </c>
+      <c r="B119" s="32">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=8)*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
+        <v/>
+      </c>
+      <c r="C119" s="32">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=8)*('Lead-Tracking 2026'!$C$4:$C$2000="Daniel")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
+        <v/>
+      </c>
+      <c r="D119" s="32">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=8)*('Lead-Tracking 2026'!$C$4:$C$2000="Jonas")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
+        <v/>
+      </c>
+      <c r="E119" s="32">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=8)*('Lead-Tracking 2026'!$C$4:$C$2000="Angie")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
+        <v/>
+      </c>
+      <c r="F119" s="32">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=8)*('Lead-Tracking 2026'!$C$4:$C$2000="Norbert")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
+        <v/>
+      </c>
+      <c r="G119" s="32">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=8)*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
+        <v/>
+      </c>
+      <c r="H119" s="32">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=8)*('Lead-Tracking 2026'!$C$4:$C$2000="Daniel")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
+        <v/>
+      </c>
+      <c r="I119" s="32">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=8)*('Lead-Tracking 2026'!$C$4:$C$2000="Jonas")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
+        <v/>
+      </c>
+      <c r="J119" s="32">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=8)*('Lead-Tracking 2026'!$C$4:$C$2000="Angie")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
+        <v/>
+      </c>
+      <c r="K119" s="32">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=8)*('Lead-Tracking 2026'!$C$4:$C$2000="Norbert")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
+        <v/>
+      </c>
+      <c r="L119" s="32">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=8)*('Lead-Tracking 2026'!$A$4:$A$2000&lt;&gt;""))</f>
+        <v/>
+      </c>
+      <c r="M119" s="32">
+        <f>M118+B119</f>
+        <v/>
+      </c>
+    </row>
+    <row r="120" ht="18" customHeight="1">
+      <c r="A120" s="29" t="inlineStr">
+        <is>
+          <t>September</t>
+        </is>
+      </c>
+      <c r="B120" s="30">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=9)*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
+        <v/>
+      </c>
+      <c r="C120" s="30">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=9)*('Lead-Tracking 2026'!$C$4:$C$2000="Daniel")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
+        <v/>
+      </c>
+      <c r="D120" s="30">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=9)*('Lead-Tracking 2026'!$C$4:$C$2000="Jonas")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
+        <v/>
+      </c>
+      <c r="E120" s="30">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=9)*('Lead-Tracking 2026'!$C$4:$C$2000="Angie")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
+        <v/>
+      </c>
+      <c r="F120" s="30">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=9)*('Lead-Tracking 2026'!$C$4:$C$2000="Norbert")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
+        <v/>
+      </c>
+      <c r="G120" s="30">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=9)*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
+        <v/>
+      </c>
+      <c r="H120" s="30">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=9)*('Lead-Tracking 2026'!$C$4:$C$2000="Daniel")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
+        <v/>
+      </c>
+      <c r="I120" s="30">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=9)*('Lead-Tracking 2026'!$C$4:$C$2000="Jonas")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
+        <v/>
+      </c>
+      <c r="J120" s="30">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=9)*('Lead-Tracking 2026'!$C$4:$C$2000="Angie")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
+        <v/>
+      </c>
+      <c r="K120" s="30">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=9)*('Lead-Tracking 2026'!$C$4:$C$2000="Norbert")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
+        <v/>
+      </c>
+      <c r="L120" s="30">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=9)*('Lead-Tracking 2026'!$A$4:$A$2000&lt;&gt;""))</f>
+        <v/>
+      </c>
+      <c r="M120" s="30">
+        <f>M119+B120</f>
+        <v/>
+      </c>
+    </row>
+    <row r="121" ht="18" customHeight="1">
+      <c r="A121" s="31" t="inlineStr">
+        <is>
+          <t>Oktober</t>
+        </is>
+      </c>
+      <c r="B121" s="32">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=10)*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
+        <v/>
+      </c>
+      <c r="C121" s="32">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=10)*('Lead-Tracking 2026'!$C$4:$C$2000="Daniel")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
+        <v/>
+      </c>
+      <c r="D121" s="32">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=10)*('Lead-Tracking 2026'!$C$4:$C$2000="Jonas")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
+        <v/>
+      </c>
+      <c r="E121" s="32">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=10)*('Lead-Tracking 2026'!$C$4:$C$2000="Angie")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
+        <v/>
+      </c>
+      <c r="F121" s="32">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=10)*('Lead-Tracking 2026'!$C$4:$C$2000="Norbert")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
+        <v/>
+      </c>
+      <c r="G121" s="32">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=10)*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
+        <v/>
+      </c>
+      <c r="H121" s="32">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=10)*('Lead-Tracking 2026'!$C$4:$C$2000="Daniel")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
+        <v/>
+      </c>
+      <c r="I121" s="32">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=10)*('Lead-Tracking 2026'!$C$4:$C$2000="Jonas")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
+        <v/>
+      </c>
+      <c r="J121" s="32">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=10)*('Lead-Tracking 2026'!$C$4:$C$2000="Angie")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
+        <v/>
+      </c>
+      <c r="K121" s="32">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=10)*('Lead-Tracking 2026'!$C$4:$C$2000="Norbert")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
+        <v/>
+      </c>
+      <c r="L121" s="32">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=10)*('Lead-Tracking 2026'!$A$4:$A$2000&lt;&gt;""))</f>
+        <v/>
+      </c>
+      <c r="M121" s="32">
+        <f>M120+B121</f>
+        <v/>
+      </c>
+    </row>
+    <row r="122" ht="18" customHeight="1">
+      <c r="A122" s="29" t="inlineStr">
+        <is>
+          <t>November</t>
+        </is>
+      </c>
+      <c r="B122" s="30">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=11)*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
+        <v/>
+      </c>
+      <c r="C122" s="30">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=11)*('Lead-Tracking 2026'!$C$4:$C$2000="Daniel")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
+        <v/>
+      </c>
+      <c r="D122" s="30">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=11)*('Lead-Tracking 2026'!$C$4:$C$2000="Jonas")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
+        <v/>
+      </c>
+      <c r="E122" s="30">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=11)*('Lead-Tracking 2026'!$C$4:$C$2000="Angie")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
+        <v/>
+      </c>
+      <c r="F122" s="30">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=11)*('Lead-Tracking 2026'!$C$4:$C$2000="Norbert")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
+        <v/>
+      </c>
+      <c r="G122" s="30">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=11)*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
+        <v/>
+      </c>
+      <c r="H122" s="30">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=11)*('Lead-Tracking 2026'!$C$4:$C$2000="Daniel")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
+        <v/>
+      </c>
+      <c r="I122" s="30">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=11)*('Lead-Tracking 2026'!$C$4:$C$2000="Jonas")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
+        <v/>
+      </c>
+      <c r="J122" s="30">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=11)*('Lead-Tracking 2026'!$C$4:$C$2000="Angie")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
+        <v/>
+      </c>
+      <c r="K122" s="30">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=11)*('Lead-Tracking 2026'!$C$4:$C$2000="Norbert")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
+        <v/>
+      </c>
+      <c r="L122" s="30">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=11)*('Lead-Tracking 2026'!$A$4:$A$2000&lt;&gt;""))</f>
+        <v/>
+      </c>
+      <c r="M122" s="30">
+        <f>M121+B122</f>
+        <v/>
+      </c>
+    </row>
+    <row r="123" ht="18" customHeight="1">
+      <c r="A123" s="31" t="inlineStr">
+        <is>
+          <t>Dezember</t>
+        </is>
+      </c>
+      <c r="B123" s="32">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=12)*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
+        <v/>
+      </c>
+      <c r="C123" s="32">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=12)*('Lead-Tracking 2026'!$C$4:$C$2000="Daniel")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
+        <v/>
+      </c>
+      <c r="D123" s="32">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=12)*('Lead-Tracking 2026'!$C$4:$C$2000="Jonas")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
+        <v/>
+      </c>
+      <c r="E123" s="32">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=12)*('Lead-Tracking 2026'!$C$4:$C$2000="Angie")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
+        <v/>
+      </c>
+      <c r="F123" s="32">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=12)*('Lead-Tracking 2026'!$C$4:$C$2000="Norbert")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
+        <v/>
+      </c>
+      <c r="G123" s="32">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=12)*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
+        <v/>
+      </c>
+      <c r="H123" s="32">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=12)*('Lead-Tracking 2026'!$C$4:$C$2000="Daniel")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
+        <v/>
+      </c>
+      <c r="I123" s="32">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=12)*('Lead-Tracking 2026'!$C$4:$C$2000="Jonas")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
+        <v/>
+      </c>
+      <c r="J123" s="32">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=12)*('Lead-Tracking 2026'!$C$4:$C$2000="Angie")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
+        <v/>
+      </c>
+      <c r="K123" s="32">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=12)*('Lead-Tracking 2026'!$C$4:$C$2000="Norbert")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
+        <v/>
+      </c>
+      <c r="L123" s="32">
+        <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=12)*('Lead-Tracking 2026'!$A$4:$A$2000&lt;&gt;""))</f>
+        <v/>
+      </c>
+      <c r="M123" s="32">
+        <f>M122+B123</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="A3:F3"/>
+  <mergeCells count="7">
+    <mergeCell ref="A24:F24"/>
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A16:F16"/>
+    <mergeCell ref="A110:M110"/>
     <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A3:F3"/>
+    <mergeCell ref="A25:F25"/>
   </mergeCells>
   <conditionalFormatting sqref="B14:F14">
     <cfRule type="expression" priority="1" dxfId="11">
@@ -6518,6 +7842,7 @@
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -6557,17 +7882,17 @@
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="27" t="inlineStr">
+      <c r="A5" s="33" t="inlineStr">
         <is>
           <t>Kuerzel</t>
         </is>
       </c>
-      <c r="B5" s="27" t="inlineStr">
+      <c r="B5" s="33" t="inlineStr">
         <is>
           <t>Beschreibung</t>
         </is>
       </c>
-      <c r="C5" s="27" t="inlineStr">
+      <c r="C5" s="33" t="inlineStr">
         <is>
           <t>Strategie</t>
         </is>
@@ -6751,17 +8076,17 @@
       </c>
     </row>
     <row r="18" ht="20" customHeight="1">
-      <c r="A18" s="27" t="inlineStr">
+      <c r="A18" s="33" t="inlineStr">
         <is>
           <t>Code</t>
         </is>
       </c>
-      <c r="B18" s="27" t="inlineStr">
+      <c r="B18" s="33" t="inlineStr">
         <is>
           <t>Kunden-Formulierung / Bedeutung</t>
         </is>
       </c>
-      <c r="C18" s="27" t="inlineStr">
+      <c r="C18" s="33" t="inlineStr">
         <is>
           <t>Naechster Schritt</t>
         </is>
@@ -6945,48 +8270,48 @@
       </c>
     </row>
     <row r="31" ht="18" customHeight="1">
-      <c r="A31" s="28" t="inlineStr">
+      <c r="A31" s="34" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
       </c>
-      <c r="B31" s="29" t="inlineStr">
+      <c r="B31" s="35" t="inlineStr">
         <is>
           <t>Check-Datum liegt in &gt; 2 Tagen – alles im Plan</t>
         </is>
       </c>
     </row>
     <row r="32" ht="18" customHeight="1">
-      <c r="A32" s="30" t="inlineStr">
+      <c r="A32" s="36" t="inlineStr">
         <is>
           <t>~</t>
         </is>
       </c>
-      <c r="B32" s="31" t="inlineStr">
+      <c r="B32" s="37" t="inlineStr">
         <is>
           <t>Check-Datum heute oder morgen – sofort handeln</t>
         </is>
       </c>
     </row>
     <row r="33" ht="18" customHeight="1">
-      <c r="A33" s="32" t="inlineStr">
+      <c r="A33" s="38" t="inlineStr">
         <is>
           <t>!</t>
         </is>
       </c>
-      <c r="B33" s="33" t="inlineStr">
+      <c r="B33" s="39" t="inlineStr">
         <is>
           <t>Check-Datum ueberschritten – dringend nachfassen!</t>
         </is>
       </c>
     </row>
     <row r="34" ht="18" customHeight="1">
-      <c r="A34" s="34" t="inlineStr">
+      <c r="A34" s="40" t="inlineStr">
         <is>
           <t>o</t>
         </is>
       </c>
-      <c r="B34" s="35" t="inlineStr">
+      <c r="B34" s="41" t="inlineStr">
         <is>
           <t>Abgeschlossen / Verloren / Wartet – kein Follow-up</t>
         </is>
@@ -7000,72 +8325,72 @@
       </c>
     </row>
     <row r="37" ht="18" customHeight="1">
-      <c r="A37" s="36" t="inlineStr">
+      <c r="A37" s="42" t="inlineStr">
         <is>
           <t>Kauf abgeschlossen</t>
         </is>
       </c>
-      <c r="B37" s="29" t="inlineStr">
+      <c r="B37" s="35" t="inlineStr">
         <is>
           <t>Abgeschlossen, kein Follow-up</t>
         </is>
       </c>
     </row>
     <row r="38" ht="18" customHeight="1">
-      <c r="A38" s="37" t="inlineStr">
+      <c r="A38" s="43" t="inlineStr">
         <is>
           <t>Heimcheck angelegt</t>
         </is>
       </c>
-      <c r="B38" s="38" t="inlineStr">
+      <c r="B38" s="44" t="inlineStr">
         <is>
           <t>Naechster Schritt: Check-Anruf</t>
         </is>
       </c>
     </row>
     <row r="39" ht="18" customHeight="1">
-      <c r="A39" s="39" t="inlineStr">
+      <c r="A39" s="45" t="inlineStr">
         <is>
           <t>Entscheidungscheck geplant</t>
         </is>
       </c>
-      <c r="B39" s="31" t="inlineStr">
+      <c r="B39" s="37" t="inlineStr">
         <is>
           <t>Kurz vor Abschluss – nachfassen</t>
         </is>
       </c>
     </row>
     <row r="40" ht="18" customHeight="1">
-      <c r="A40" s="40" t="inlineStr">
+      <c r="A40" s="46" t="inlineStr">
         <is>
           <t>Angebot konkret</t>
         </is>
       </c>
-      <c r="B40" s="41" t="inlineStr">
+      <c r="B40" s="47" t="inlineStr">
         <is>
           <t>Angebot liegt vor</t>
         </is>
       </c>
     </row>
     <row r="41" ht="18" customHeight="1">
-      <c r="A41" s="42" t="inlineStr">
+      <c r="A41" s="48" t="inlineStr">
         <is>
           <t>Verloren</t>
         </is>
       </c>
-      <c r="B41" s="33" t="inlineStr">
+      <c r="B41" s="39" t="inlineStr">
         <is>
           <t>Lead verloren – Verlustgrund eintragen</t>
         </is>
       </c>
     </row>
     <row r="42" ht="18" customHeight="1">
-      <c r="A42" s="43" t="inlineStr">
+      <c r="A42" s="49" t="inlineStr">
         <is>
           <t>Warten auf Raum</t>
         </is>
       </c>
-      <c r="B42" s="35" t="inlineStr">
+      <c r="B42" s="41" t="inlineStr">
         <is>
           <t>Wiedervorlage in Monaten</t>
         </is>

</xml_diff>

<commit_message>
Fix Abschlussquote coloring + add Abschluss traffic lights
- Bug: Abschlussquote turned green for any number (ISNUMBER only). Replaced
  with real gates: <40% rot, 40-60% gelb, >60% gruen; ISNUMBER guard keeps
  empty "—" uncolored
- Abschluss column (Lead-Tracking): Ja=gruen, Nein=rot, Offen=gelb
- Legende: added Abschluss-Ampel and Abschlussquote-Gates reference sections

https://claude.ai/code/session_01WiRUeJ8tQNpk2kLkUtpvQn
</commit_message>
<xml_diff>
--- a/fitshop-sop/Fitshop_Tracking_2026.xlsx
+++ b/fitshop-sop/Fitshop_Tracking_2026.xlsx
@@ -219,7 +219,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="50">
+  <cellXfs count="53">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -328,11 +328,20 @@
     <xf numFmtId="0" fontId="5" fillId="11" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="8" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="9" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="13">
+  <dxfs count="14">
     <dxf>
       <font>
         <name val="Calibri"/>
@@ -507,6 +516,20 @@
         <patternFill patternType="solid">
           <fgColor rgb="00C8E6C9"/>
           <bgColor rgb="00C8E6C9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Calibri"/>
+        <b val="1"/>
+        <color rgb="00F57F17"/>
+        <sz val="10"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FFF9C4"/>
+          <bgColor rgb="00FFF9C4"/>
         </patternFill>
       </fill>
     </dxf>
@@ -6615,6 +6638,17 @@
       <formula>L4&lt;=2</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="Q4:Q2000">
+    <cfRule type="expression" priority="16" dxfId="7">
+      <formula>Q4="Ja"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="17" dxfId="6">
+      <formula>Q4="Nein"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="18" dxfId="3">
+      <formula>Q4="Offen"</formula>
+    </cfRule>
+  </conditionalFormatting>
   <dataValidations count="9">
     <dataValidation sqref="C4:C2000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Daniel,Jonas,Angie,Norbert"</formula1>
@@ -7838,7 +7872,13 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="B7:F7">
     <cfRule type="expression" priority="2" dxfId="12">
-      <formula>ISNUMBER(B7)</formula>
+      <formula>AND(ISNUMBER(B7),B7&gt;=0.6)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="3" dxfId="13">
+      <formula>AND(ISNUMBER(B7),B7&gt;=0.4,B7&lt;0.6)</formula>
+    </cfRule>
+    <cfRule type="expression" priority="4" dxfId="11">
+      <formula>AND(ISNUMBER(B7),B7&lt;0.4)</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -7852,7 +7892,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C42"/>
+  <dimension ref="A1:C53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -8396,24 +8436,118 @@
         </is>
       </c>
     </row>
+    <row r="44" ht="22" customHeight="1">
+      <c r="A44" s="20" t="inlineStr">
+        <is>
+          <t>ABSCHLUSS-AMPEL (Spalte Abschluss)</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="18" customHeight="1">
+      <c r="A45" s="50" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="B45" s="35" t="inlineStr">
+        <is>
+          <t>Verkauf abgeschlossen</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="18" customHeight="1">
+      <c r="A46" s="51" t="inlineStr">
+        <is>
+          <t>Offen</t>
+        </is>
+      </c>
+      <c r="B46" s="37" t="inlineStr">
+        <is>
+          <t>Lead laeuft noch – dranbleiben</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="18" customHeight="1">
+      <c r="A47" s="52" t="inlineStr">
+        <is>
+          <t>Nein</t>
+        </is>
+      </c>
+      <c r="B47" s="39" t="inlineStr">
+        <is>
+          <t>Lead verloren – Verlustgrund eintragen</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="22" customHeight="1">
+      <c r="A50" s="20" t="inlineStr">
+        <is>
+          <t>ABSCHLUSSQUOTE-GATES (KPI Dashboard)</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="18" customHeight="1">
+      <c r="A51" s="50" t="inlineStr">
+        <is>
+          <t>&gt; 60 %</t>
+        </is>
+      </c>
+      <c r="B51" s="35" t="inlineStr">
+        <is>
+          <t>Top – Ziel uebertroffen</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="18" customHeight="1">
+      <c r="A52" s="51" t="inlineStr">
+        <is>
+          <t>40 – 60 %</t>
+        </is>
+      </c>
+      <c r="B52" s="37" t="inlineStr">
+        <is>
+          <t>Solide – im Zielkorridor</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="18" customHeight="1">
+      <c r="A53" s="52" t="inlineStr">
+        <is>
+          <t>&lt; 40 %</t>
+        </is>
+      </c>
+      <c r="B53" s="39" t="inlineStr">
+        <is>
+          <t>Unter Soll – Prozess pruefen</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="16">
+  <mergeCells count="24">
+    <mergeCell ref="B47:C47"/>
+    <mergeCell ref="B46:C46"/>
+    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="A50:C50"/>
+    <mergeCell ref="A2:C2"/>
     <mergeCell ref="B39:C39"/>
+    <mergeCell ref="B52:C52"/>
+    <mergeCell ref="B42:C42"/>
+    <mergeCell ref="A17:C17"/>
+    <mergeCell ref="A4:C4"/>
+    <mergeCell ref="B53:C53"/>
     <mergeCell ref="B38:C38"/>
+    <mergeCell ref="A44:C44"/>
+    <mergeCell ref="B34:C34"/>
+    <mergeCell ref="B37:C37"/>
+    <mergeCell ref="A30:C30"/>
+    <mergeCell ref="B40:C40"/>
     <mergeCell ref="A36:C36"/>
     <mergeCell ref="B33:C33"/>
     <mergeCell ref="A1:C1"/>
-    <mergeCell ref="B34:C34"/>
-    <mergeCell ref="B37:C37"/>
-    <mergeCell ref="B42:C42"/>
-    <mergeCell ref="A17:C17"/>
+    <mergeCell ref="B51:C51"/>
+    <mergeCell ref="B45:C45"/>
     <mergeCell ref="B32:C32"/>
-    <mergeCell ref="A30:C30"/>
-    <mergeCell ref="B31:C31"/>
-    <mergeCell ref="B40:C40"/>
     <mergeCell ref="B41:C41"/>
-    <mergeCell ref="A4:C4"/>
-    <mergeCell ref="A2:C2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fix 4 chart XML bugs found in structural audit
- BUG-1: catAx axPos was 'l' (left) instead of 'b' (bottom) on both charts,
  which causes LibreOffice to render column charts sideways
- BUG-2: category axis used numRef for text month names (Jan-Dez) instead of
  strRef; fixed via AxDataSource(strRef=StrRef()) override after add_data()
- BUG-3: secondary Y-axis (cumulative line, id=200) had axPos='l', causing
  overlap with the primary axis; corrected to axPos='r' (right side)
- BUG-4: no numFmt on value axes; primary axes now show #,##0 (EUR with
  thousands separator), secondary axis shows integer counts

https://claude.ai/code/session_01WiRUeJ8tQNpk2kLkUtpvQn
</commit_message>
<xml_diff>
--- a/fitshop-sop/Fitshop_Tracking_2026.xlsx
+++ b/fitshop-sop/Fitshop_Tracking_2026.xlsx
@@ -649,9 +649,9 @@
             </a:ln>
           </spPr>
           <cat>
-            <numRef>
+            <strRef>
               <f>'KPI Dashboard'!$A$112:$A$123</f>
-            </numRef>
+            </strRef>
           </cat>
           <val>
             <numRef>
@@ -679,9 +679,9 @@
             </a:ln>
           </spPr>
           <cat>
-            <numRef>
+            <strRef>
               <f>'KPI Dashboard'!$A$112:$A$123</f>
-            </numRef>
+            </strRef>
           </cat>
           <val>
             <numRef>
@@ -709,9 +709,9 @@
             </a:ln>
           </spPr>
           <cat>
-            <numRef>
+            <strRef>
               <f>'KPI Dashboard'!$A$112:$A$123</f>
-            </numRef>
+            </strRef>
           </cat>
           <val>
             <numRef>
@@ -739,9 +739,9 @@
             </a:ln>
           </spPr>
           <cat>
-            <numRef>
+            <strRef>
               <f>'KPI Dashboard'!$A$112:$A$123</f>
-            </numRef>
+            </strRef>
           </cat>
           <val>
             <numRef>
@@ -788,9 +788,9 @@
             </spPr>
           </marker>
           <cat>
-            <numRef>
+            <strRef>
               <f>'KPI Dashboard'!$A$112:$A$123</f>
-            </numRef>
+            </strRef>
           </cat>
           <val>
             <numRef>
@@ -807,7 +807,7 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
-        <axPos val="l"/>
+        <axPos val="b"/>
         <title>
           <tx>
             <rich>
@@ -850,6 +850,7 @@
             </rich>
           </tx>
         </title>
+        <numFmt formatCode="#,##0" sourceLinked="0"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="10"/>
@@ -859,7 +860,7 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
-        <axPos val="l"/>
+        <axPos val="r"/>
         <majorGridlines/>
         <title>
           <tx>
@@ -876,6 +877,7 @@
             </rich>
           </tx>
         </title>
+        <numFmt formatCode="#,##0" sourceLinked="0"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="10"/>
@@ -934,9 +936,9 @@
             </a:ln>
           </spPr>
           <cat>
-            <numRef>
+            <strRef>
               <f>'KPI Dashboard'!$A$112:$A$123</f>
-            </numRef>
+            </strRef>
           </cat>
           <val>
             <numRef>
@@ -964,9 +966,9 @@
             </a:ln>
           </spPr>
           <cat>
-            <numRef>
+            <strRef>
               <f>'KPI Dashboard'!$A$112:$A$123</f>
-            </numRef>
+            </strRef>
           </cat>
           <val>
             <numRef>
@@ -994,9 +996,9 @@
             </a:ln>
           </spPr>
           <cat>
-            <numRef>
+            <strRef>
               <f>'KPI Dashboard'!$A$112:$A$123</f>
-            </numRef>
+            </strRef>
           </cat>
           <val>
             <numRef>
@@ -1024,9 +1026,9 @@
             </a:ln>
           </spPr>
           <cat>
-            <numRef>
+            <strRef>
               <f>'KPI Dashboard'!$A$112:$A$123</f>
-            </numRef>
+            </strRef>
           </cat>
           <val>
             <numRef>
@@ -1043,7 +1045,7 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
-        <axPos val="l"/>
+        <axPos val="b"/>
         <title>
           <tx>
             <rich>
@@ -1086,6 +1088,7 @@
             </rich>
           </tx>
         </title>
+        <numFmt formatCode="0" sourceLinked="0"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="10"/>

</xml_diff>

<commit_message>
Split combo chart into separate charts for Google Sheets compatibility
Google Sheets cannot import Excel combo charts (barChart+lineChart in one
plotArea). Replaced with 3 independent charts:
- Chart 1a: Stacked BarChart (Umsatz per MA per month, 4 series)
- Chart 1b: LineChart (kumulierter Umsatz Gesamttrend, Fitshop-red line)
- Chart 2:  Clustered BarChart (Abschluesse per MA per month, unchanged)

https://claude.ai/code/session_01WiRUeJ8tQNpk2kLkUtpvQn
</commit_message>
<xml_diff>
--- a/fitshop-sop/Fitshop_Tracking_2026.xlsx
+++ b/fitshop-sop/Fitshop_Tracking_2026.xlsx
@@ -754,54 +754,6 @@
         <axId val="10"/>
         <axId val="100"/>
       </barChart>
-      <lineChart>
-        <grouping val="standard"/>
-        <ser>
-          <idx val="4"/>
-          <order val="4"/>
-          <tx>
-            <strRef>
-              <f>'KPI Dashboard'!M111</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:ln w="31750">
-              <a:solidFill>
-                <a:srgbClr val="2D2D2D"/>
-              </a:solidFill>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="circle"/>
-            <size val="6"/>
-            <spPr>
-              <a:solidFill>
-                <a:srgbClr val="2D2D2D"/>
-              </a:solidFill>
-              <a:ln>
-                <a:solidFill>
-                  <a:srgbClr val="2D2D2D"/>
-                </a:solidFill>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <strRef>
-              <f>'KPI Dashboard'!$A$112:$A$123</f>
-            </strRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'KPI Dashboard'!$M$112:$M$123</f>
-            </numRef>
-          </val>
-          <smooth val="1"/>
-        </ser>
-        <axId val="10"/>
-        <axId val="200"/>
-      </lineChart>
       <catAx>
         <axId val="10"/>
         <scaling>
@@ -855,12 +807,116 @@
         <minorTickMark val="none"/>
         <crossAx val="10"/>
       </valAx>
-      <valAx>
-        <axId val="200"/>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="10"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Kumulierter Umsatz 2026 – Gesamttrend (EUR)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'KPI Dashboard'!M111</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln w="31750">
+              <a:solidFill>
+                <a:srgbClr val="E31E24"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="circle"/>
+            <size val="6"/>
+            <spPr>
+              <a:solidFill>
+                <a:srgbClr val="E31E24"/>
+              </a:solidFill>
+              <a:ln>
+                <a:solidFill>
+                  <a:srgbClr val="E31E24"/>
+                </a:solidFill>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <strRef>
+              <f>'KPI Dashboard'!$A$112:$A$123</f>
+            </strRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'KPI Dashboard'!$M$112:$M$123</f>
+            </numRef>
+          </val>
+          <smooth val="1"/>
+        </ser>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
         <scaling>
           <orientation val="minMax"/>
         </scaling>
-        <axPos val="r"/>
+        <axPos val="b"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Monat</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
         <majorGridlines/>
         <title>
           <tx>
@@ -881,7 +937,6 @@
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="10"/>
-        <crosses val="max"/>
       </valAx>
     </plotArea>
     <legend>
@@ -893,7 +948,7 @@
 </chartSpace>
 </file>
 
-<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="10"/>
   <chart>
@@ -1112,7 +1167,7 @@
       <row>25</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="9360000" cy="5400000"/>
+    <ext cx="9360000" cy="5040000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="1" name="Chart 1"/>
@@ -1131,10 +1186,10 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>48</row>
+      <row>46</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="7920000" cy="4320000"/>
+    <ext cx="9360000" cy="3600000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="2" name="Chart 2"/>
@@ -1144,6 +1199,28 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>62</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="7920000" cy="4320000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="3" name="Chart 3"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId3"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>

</xml_diff>

<commit_message>
Replace broken openpyxl charts with native Google Apps Script
openpyxl-generated chart XML is not reliably supported by Google Sheets or
LibreOffice. Removed all embedded charts from the xlsx to eliminate errors.

Added fitshop_charts.gs: a Google Apps Script that creates 3 native Google
Sheets charts (stacked column / line / clustered column) directly via the
Sheets API. Charts reference the helper table at rows 111-123 which remains
in KPI Dashboard with all SUMPRODUCT formulas intact.

To use: Extensions > Apps Script > paste fitshop_charts.gs > run createFitshopCharts

https://claude.ai/code/session_01WiRUeJ8tQNpk2kLkUtpvQn
</commit_message>
<xml_diff>
--- a/fitshop-sop/Fitshop_Tracking_2026.xlsx
+++ b/fitshop-sop/Fitshop_Tracking_2026.xlsx
@@ -23,7 +23,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="#,##0 &quot;EUR&quot;"/>
   </numFmts>
-  <fonts count="12">
+  <fonts count="13">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -86,6 +86,12 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
+      <color rgb="00F57F17"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
       <i val="1"/>
       <color rgb="00AAAAAA"/>
       <sz val="8"/>
@@ -130,14 +136,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C8E6C9"/>
-        <bgColor rgb="00C8E6C9"/>
+        <fgColor rgb="00FFF9C4"/>
+        <bgColor rgb="00FFF9C4"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF9C4"/>
-        <bgColor rgb="00FFF9C4"/>
+        <fgColor rgb="00C8E6C9"/>
+        <bgColor rgb="00C8E6C9"/>
       </patternFill>
     </fill>
     <fill>
@@ -219,7 +225,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="53">
+  <cellXfs count="54">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -291,10 +297,13 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -304,14 +313,14 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="6" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -320,18 +329,18 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="9" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="10" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="10" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="11" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="11" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="8" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="9" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -604,629 +613,6 @@
     </indexedColors>
   </colors>
 </styleSheet>
-</file>
-
-<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="10"/>
-  <chart>
-    <title>
-      <tx>
-        <rich>
-          <a:bodyPr/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr/>
-            </a:pPr>
-            <a:r>
-              <a:t>Umsatz-Entwicklung 2026 nach Mitarbeiter (EUR)</a:t>
-            </a:r>
-          </a:p>
-        </rich>
-      </tx>
-    </title>
-    <plotArea>
-      <barChart>
-        <barDir val="col"/>
-        <grouping val="stacked"/>
-        <ser>
-          <idx val="0"/>
-          <order val="0"/>
-          <tx>
-            <strRef>
-              <f>'KPI Dashboard'!C111</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:solidFill>
-              <a:srgbClr val="E31E24"/>
-            </a:solidFill>
-            <a:ln>
-              <a:solidFill>
-                <a:srgbClr val="E31E24"/>
-              </a:solidFill>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <cat>
-            <strRef>
-              <f>'KPI Dashboard'!$A$112:$A$123</f>
-            </strRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'KPI Dashboard'!$C$112:$C$123</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="1"/>
-          <order val="1"/>
-          <tx>
-            <strRef>
-              <f>'KPI Dashboard'!D111</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:solidFill>
-              <a:srgbClr val="1565C0"/>
-            </a:solidFill>
-            <a:ln>
-              <a:solidFill>
-                <a:srgbClr val="1565C0"/>
-              </a:solidFill>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <cat>
-            <strRef>
-              <f>'KPI Dashboard'!$A$112:$A$123</f>
-            </strRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'KPI Dashboard'!$D$112:$D$123</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="2"/>
-          <order val="2"/>
-          <tx>
-            <strRef>
-              <f>'KPI Dashboard'!E111</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:solidFill>
-              <a:srgbClr val="2E7D32"/>
-            </a:solidFill>
-            <a:ln>
-              <a:solidFill>
-                <a:srgbClr val="2E7D32"/>
-              </a:solidFill>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <cat>
-            <strRef>
-              <f>'KPI Dashboard'!$A$112:$A$123</f>
-            </strRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'KPI Dashboard'!$E$112:$E$123</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="3"/>
-          <order val="3"/>
-          <tx>
-            <strRef>
-              <f>'KPI Dashboard'!F111</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:solidFill>
-              <a:srgbClr val="E65100"/>
-            </a:solidFill>
-            <a:ln>
-              <a:solidFill>
-                <a:srgbClr val="E65100"/>
-              </a:solidFill>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <cat>
-            <strRef>
-              <f>'KPI Dashboard'!$A$112:$A$123</f>
-            </strRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'KPI Dashboard'!$F$112:$F$123</f>
-            </numRef>
-          </val>
-        </ser>
-        <gapWidth val="150"/>
-        <overlap val="100"/>
-        <axId val="10"/>
-        <axId val="100"/>
-      </barChart>
-      <catAx>
-        <axId val="10"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <axPos val="b"/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>Monat</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="100"/>
-        <lblOffset val="100"/>
-      </catAx>
-      <valAx>
-        <axId val="100"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <axPos val="l"/>
-        <majorGridlines/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>EUR (monatlich)</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
-        <numFmt formatCode="#,##0" sourceLinked="0"/>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="10"/>
-      </valAx>
-    </plotArea>
-    <legend>
-      <legendPos val="r"/>
-    </legend>
-    <plotVisOnly val="1"/>
-    <dispBlanksAs val="gap"/>
-  </chart>
-</chartSpace>
-</file>
-
-<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="10"/>
-  <chart>
-    <title>
-      <tx>
-        <rich>
-          <a:bodyPr/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr/>
-            </a:pPr>
-            <a:r>
-              <a:t>Kumulierter Umsatz 2026 – Gesamttrend (EUR)</a:t>
-            </a:r>
-          </a:p>
-        </rich>
-      </tx>
-    </title>
-    <plotArea>
-      <lineChart>
-        <grouping val="standard"/>
-        <ser>
-          <idx val="0"/>
-          <order val="0"/>
-          <tx>
-            <strRef>
-              <f>'KPI Dashboard'!M111</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:ln w="31750">
-              <a:solidFill>
-                <a:srgbClr val="E31E24"/>
-              </a:solidFill>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="circle"/>
-            <size val="6"/>
-            <spPr>
-              <a:solidFill>
-                <a:srgbClr val="E31E24"/>
-              </a:solidFill>
-              <a:ln>
-                <a:solidFill>
-                  <a:srgbClr val="E31E24"/>
-                </a:solidFill>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <cat>
-            <strRef>
-              <f>'KPI Dashboard'!$A$112:$A$123</f>
-            </strRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'KPI Dashboard'!$M$112:$M$123</f>
-            </numRef>
-          </val>
-          <smooth val="1"/>
-        </ser>
-        <axId val="10"/>
-        <axId val="100"/>
-      </lineChart>
-      <catAx>
-        <axId val="10"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <axPos val="b"/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>Monat</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="100"/>
-        <lblOffset val="100"/>
-      </catAx>
-      <valAx>
-        <axId val="100"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <axPos val="l"/>
-        <majorGridlines/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>Kumuliert (EUR)</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
-        <numFmt formatCode="#,##0" sourceLinked="0"/>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="10"/>
-      </valAx>
-    </plotArea>
-    <legend>
-      <legendPos val="r"/>
-    </legend>
-    <plotVisOnly val="1"/>
-    <dispBlanksAs val="gap"/>
-  </chart>
-</chartSpace>
-</file>
-
-<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="10"/>
-  <chart>
-    <title>
-      <tx>
-        <rich>
-          <a:bodyPr/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr/>
-            </a:pPr>
-            <a:r>
-              <a:t>Abschlüsse pro Monat nach Mitarbeiter</a:t>
-            </a:r>
-          </a:p>
-        </rich>
-      </tx>
-    </title>
-    <plotArea>
-      <barChart>
-        <barDir val="col"/>
-        <grouping val="clustered"/>
-        <ser>
-          <idx val="0"/>
-          <order val="0"/>
-          <tx>
-            <strRef>
-              <f>'KPI Dashboard'!H111</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:solidFill>
-              <a:srgbClr val="E31E24"/>
-            </a:solidFill>
-            <a:ln>
-              <a:solidFill>
-                <a:srgbClr val="E31E24"/>
-              </a:solidFill>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <cat>
-            <strRef>
-              <f>'KPI Dashboard'!$A$112:$A$123</f>
-            </strRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'KPI Dashboard'!$H$112:$H$123</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="1"/>
-          <order val="1"/>
-          <tx>
-            <strRef>
-              <f>'KPI Dashboard'!I111</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:solidFill>
-              <a:srgbClr val="1565C0"/>
-            </a:solidFill>
-            <a:ln>
-              <a:solidFill>
-                <a:srgbClr val="1565C0"/>
-              </a:solidFill>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <cat>
-            <strRef>
-              <f>'KPI Dashboard'!$A$112:$A$123</f>
-            </strRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'KPI Dashboard'!$I$112:$I$123</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="2"/>
-          <order val="2"/>
-          <tx>
-            <strRef>
-              <f>'KPI Dashboard'!J111</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:solidFill>
-              <a:srgbClr val="2E7D32"/>
-            </a:solidFill>
-            <a:ln>
-              <a:solidFill>
-                <a:srgbClr val="2E7D32"/>
-              </a:solidFill>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <cat>
-            <strRef>
-              <f>'KPI Dashboard'!$A$112:$A$123</f>
-            </strRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'KPI Dashboard'!$J$112:$J$123</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="3"/>
-          <order val="3"/>
-          <tx>
-            <strRef>
-              <f>'KPI Dashboard'!K111</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:solidFill>
-              <a:srgbClr val="E65100"/>
-            </a:solidFill>
-            <a:ln>
-              <a:solidFill>
-                <a:srgbClr val="E65100"/>
-              </a:solidFill>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <cat>
-            <strRef>
-              <f>'KPI Dashboard'!$A$112:$A$123</f>
-            </strRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'KPI Dashboard'!$K$112:$K$123</f>
-            </numRef>
-          </val>
-        </ser>
-        <gapWidth val="150"/>
-        <axId val="10"/>
-        <axId val="100"/>
-      </barChart>
-      <catAx>
-        <axId val="10"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <axPos val="b"/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>Monat</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="100"/>
-        <lblOffset val="100"/>
-      </catAx>
-      <valAx>
-        <axId val="100"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <axPos val="l"/>
-        <majorGridlines/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>Anzahl Abschlüsse</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
-        <numFmt formatCode="0" sourceLinked="0"/>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="10"/>
-      </valAx>
-    </plotArea>
-    <legend>
-      <legendPos val="r"/>
-    </legend>
-    <plotVisOnly val="1"/>
-    <dispBlanksAs val="gap"/>
-  </chart>
-</chartSpace>
-</file>
-
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <oneCellAnchor>
-    <from>
-      <col>0</col>
-      <colOff>0</colOff>
-      <row>25</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="9360000" cy="5040000"/>
-    <graphicFrame>
-      <nvGraphicFramePr>
-        <cNvPr id="1" name="Chart 1"/>
-        <cNvGraphicFramePr/>
-      </nvGraphicFramePr>
-      <xfrm/>
-      <a:graphic>
-        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
-        </a:graphicData>
-      </a:graphic>
-    </graphicFrame>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>0</col>
-      <colOff>0</colOff>
-      <row>46</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="9360000" cy="3600000"/>
-    <graphicFrame>
-      <nvGraphicFramePr>
-        <cNvPr id="2" name="Chart 2"/>
-        <cNvGraphicFramePr/>
-      </nvGraphicFramePr>
-      <xfrm/>
-      <a:graphic>
-        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId2"/>
-        </a:graphicData>
-      </a:graphic>
-    </graphicFrame>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>0</col>
-      <colOff>0</colOff>
-      <row>62</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="7920000" cy="4320000"/>
-    <graphicFrame>
-      <nvGraphicFramePr>
-        <cNvPr id="3" name="Chart 3"/>
-        <cNvGraphicFramePr/>
-      </nvGraphicFramePr>
-      <xfrm/>
-      <a:graphic>
-        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId3"/>
-        </a:graphicData>
-      </a:graphic>
-    </graphicFrame>
-    <clientData/>
-  </oneCellAnchor>
-</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -7194,743 +6580,743 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="15" customHeight="1">
-      <c r="A25" s="10" t="inlineStr">
-        <is>
-          <t>Daten werden automatisch aus dem Lead-Tracking gezogen. Ansicht aktualisieren: Strg+Alt+F9</t>
+    <row r="25" ht="18" customHeight="1">
+      <c r="A25" s="27" t="inlineStr">
+        <is>
+          <t>► Diagramme erstellen: Erweiterungen → Apps Script → fitshop_charts.gs einfügen → Funktion createFitshopCharts ausführen</t>
         </is>
       </c>
     </row>
     <row r="110" ht="16" customHeight="1">
-      <c r="A110" s="27" t="inlineStr">
+      <c r="A110" s="28" t="inlineStr">
         <is>
           <t>CHART-DATEN (automatisch berechnet – nicht bearbeiten)</t>
         </is>
       </c>
     </row>
     <row r="111" ht="20" customHeight="1">
-      <c r="A111" s="28" t="inlineStr">
+      <c r="A111" s="29" t="inlineStr">
         <is>
           <t>Monat</t>
         </is>
       </c>
-      <c r="B111" s="28" t="inlineStr">
+      <c r="B111" s="29" t="inlineStr">
         <is>
           <t>Umsatz Ges.</t>
         </is>
       </c>
-      <c r="C111" s="28" t="inlineStr">
+      <c r="C111" s="29" t="inlineStr">
         <is>
           <t>Daniel EUR</t>
         </is>
       </c>
-      <c r="D111" s="28" t="inlineStr">
+      <c r="D111" s="29" t="inlineStr">
         <is>
           <t>Jonas EUR</t>
         </is>
       </c>
-      <c r="E111" s="28" t="inlineStr">
+      <c r="E111" s="29" t="inlineStr">
         <is>
           <t>Angie EUR</t>
         </is>
       </c>
-      <c r="F111" s="28" t="inlineStr">
+      <c r="F111" s="29" t="inlineStr">
         <is>
           <t>Norbert EUR</t>
         </is>
       </c>
-      <c r="G111" s="28" t="inlineStr">
+      <c r="G111" s="29" t="inlineStr">
         <is>
           <t>Abschl. Ges.</t>
         </is>
       </c>
-      <c r="H111" s="28" t="inlineStr">
+      <c r="H111" s="29" t="inlineStr">
         <is>
           <t>Daniel #</t>
         </is>
       </c>
-      <c r="I111" s="28" t="inlineStr">
+      <c r="I111" s="29" t="inlineStr">
         <is>
           <t>Jonas #</t>
         </is>
       </c>
-      <c r="J111" s="28" t="inlineStr">
+      <c r="J111" s="29" t="inlineStr">
         <is>
           <t>Angie #</t>
         </is>
       </c>
-      <c r="K111" s="28" t="inlineStr">
+      <c r="K111" s="29" t="inlineStr">
         <is>
           <t>Norbert #</t>
         </is>
       </c>
-      <c r="L111" s="28" t="inlineStr">
+      <c r="L111" s="29" t="inlineStr">
         <is>
           <t>Neue Leads</t>
         </is>
       </c>
-      <c r="M111" s="28" t="inlineStr">
+      <c r="M111" s="29" t="inlineStr">
         <is>
           <t>Kum. Umsatz</t>
         </is>
       </c>
     </row>
     <row r="112" ht="18" customHeight="1">
-      <c r="A112" s="29" t="inlineStr">
+      <c r="A112" s="30" t="inlineStr">
         <is>
           <t>Januar</t>
         </is>
       </c>
-      <c r="B112" s="30">
+      <c r="B112" s="31">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=1)*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
         <v/>
       </c>
-      <c r="C112" s="30">
+      <c r="C112" s="31">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=1)*('Lead-Tracking 2026'!$C$4:$C$2000="Daniel")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
         <v/>
       </c>
-      <c r="D112" s="30">
+      <c r="D112" s="31">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=1)*('Lead-Tracking 2026'!$C$4:$C$2000="Jonas")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
         <v/>
       </c>
-      <c r="E112" s="30">
+      <c r="E112" s="31">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=1)*('Lead-Tracking 2026'!$C$4:$C$2000="Angie")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
         <v/>
       </c>
-      <c r="F112" s="30">
+      <c r="F112" s="31">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=1)*('Lead-Tracking 2026'!$C$4:$C$2000="Norbert")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
         <v/>
       </c>
-      <c r="G112" s="30">
+      <c r="G112" s="31">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=1)*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
         <v/>
       </c>
-      <c r="H112" s="30">
+      <c r="H112" s="31">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=1)*('Lead-Tracking 2026'!$C$4:$C$2000="Daniel")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
         <v/>
       </c>
-      <c r="I112" s="30">
+      <c r="I112" s="31">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=1)*('Lead-Tracking 2026'!$C$4:$C$2000="Jonas")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
         <v/>
       </c>
-      <c r="J112" s="30">
+      <c r="J112" s="31">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=1)*('Lead-Tracking 2026'!$C$4:$C$2000="Angie")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
         <v/>
       </c>
-      <c r="K112" s="30">
+      <c r="K112" s="31">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=1)*('Lead-Tracking 2026'!$C$4:$C$2000="Norbert")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
         <v/>
       </c>
-      <c r="L112" s="30">
+      <c r="L112" s="31">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=1)*('Lead-Tracking 2026'!$A$4:$A$2000&lt;&gt;""))</f>
         <v/>
       </c>
-      <c r="M112" s="30">
+      <c r="M112" s="31">
         <f>B112</f>
         <v/>
       </c>
     </row>
     <row r="113" ht="18" customHeight="1">
-      <c r="A113" s="31" t="inlineStr">
+      <c r="A113" s="32" t="inlineStr">
         <is>
           <t>Februar</t>
         </is>
       </c>
-      <c r="B113" s="32">
+      <c r="B113" s="33">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=2)*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
         <v/>
       </c>
-      <c r="C113" s="32">
+      <c r="C113" s="33">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=2)*('Lead-Tracking 2026'!$C$4:$C$2000="Daniel")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
         <v/>
       </c>
-      <c r="D113" s="32">
+      <c r="D113" s="33">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=2)*('Lead-Tracking 2026'!$C$4:$C$2000="Jonas")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
         <v/>
       </c>
-      <c r="E113" s="32">
+      <c r="E113" s="33">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=2)*('Lead-Tracking 2026'!$C$4:$C$2000="Angie")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
         <v/>
       </c>
-      <c r="F113" s="32">
+      <c r="F113" s="33">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=2)*('Lead-Tracking 2026'!$C$4:$C$2000="Norbert")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
         <v/>
       </c>
-      <c r="G113" s="32">
+      <c r="G113" s="33">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=2)*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
         <v/>
       </c>
-      <c r="H113" s="32">
+      <c r="H113" s="33">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=2)*('Lead-Tracking 2026'!$C$4:$C$2000="Daniel")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
         <v/>
       </c>
-      <c r="I113" s="32">
+      <c r="I113" s="33">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=2)*('Lead-Tracking 2026'!$C$4:$C$2000="Jonas")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
         <v/>
       </c>
-      <c r="J113" s="32">
+      <c r="J113" s="33">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=2)*('Lead-Tracking 2026'!$C$4:$C$2000="Angie")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
         <v/>
       </c>
-      <c r="K113" s="32">
+      <c r="K113" s="33">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=2)*('Lead-Tracking 2026'!$C$4:$C$2000="Norbert")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
         <v/>
       </c>
-      <c r="L113" s="32">
+      <c r="L113" s="33">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=2)*('Lead-Tracking 2026'!$A$4:$A$2000&lt;&gt;""))</f>
         <v/>
       </c>
-      <c r="M113" s="32">
+      <c r="M113" s="33">
         <f>M112+B113</f>
         <v/>
       </c>
     </row>
     <row r="114" ht="18" customHeight="1">
-      <c r="A114" s="29" t="inlineStr">
+      <c r="A114" s="30" t="inlineStr">
         <is>
           <t>März</t>
         </is>
       </c>
-      <c r="B114" s="30">
+      <c r="B114" s="31">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=3)*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
         <v/>
       </c>
-      <c r="C114" s="30">
+      <c r="C114" s="31">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=3)*('Lead-Tracking 2026'!$C$4:$C$2000="Daniel")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
         <v/>
       </c>
-      <c r="D114" s="30">
+      <c r="D114" s="31">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=3)*('Lead-Tracking 2026'!$C$4:$C$2000="Jonas")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
         <v/>
       </c>
-      <c r="E114" s="30">
+      <c r="E114" s="31">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=3)*('Lead-Tracking 2026'!$C$4:$C$2000="Angie")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
         <v/>
       </c>
-      <c r="F114" s="30">
+      <c r="F114" s="31">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=3)*('Lead-Tracking 2026'!$C$4:$C$2000="Norbert")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
         <v/>
       </c>
-      <c r="G114" s="30">
+      <c r="G114" s="31">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=3)*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
         <v/>
       </c>
-      <c r="H114" s="30">
+      <c r="H114" s="31">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=3)*('Lead-Tracking 2026'!$C$4:$C$2000="Daniel")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
         <v/>
       </c>
-      <c r="I114" s="30">
+      <c r="I114" s="31">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=3)*('Lead-Tracking 2026'!$C$4:$C$2000="Jonas")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
         <v/>
       </c>
-      <c r="J114" s="30">
+      <c r="J114" s="31">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=3)*('Lead-Tracking 2026'!$C$4:$C$2000="Angie")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
         <v/>
       </c>
-      <c r="K114" s="30">
+      <c r="K114" s="31">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=3)*('Lead-Tracking 2026'!$C$4:$C$2000="Norbert")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
         <v/>
       </c>
-      <c r="L114" s="30">
+      <c r="L114" s="31">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=3)*('Lead-Tracking 2026'!$A$4:$A$2000&lt;&gt;""))</f>
         <v/>
       </c>
-      <c r="M114" s="30">
+      <c r="M114" s="31">
         <f>M113+B114</f>
         <v/>
       </c>
     </row>
     <row r="115" ht="18" customHeight="1">
-      <c r="A115" s="31" t="inlineStr">
+      <c r="A115" s="32" t="inlineStr">
         <is>
           <t>April</t>
         </is>
       </c>
-      <c r="B115" s="32">
+      <c r="B115" s="33">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=4)*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
         <v/>
       </c>
-      <c r="C115" s="32">
+      <c r="C115" s="33">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=4)*('Lead-Tracking 2026'!$C$4:$C$2000="Daniel")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
         <v/>
       </c>
-      <c r="D115" s="32">
+      <c r="D115" s="33">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=4)*('Lead-Tracking 2026'!$C$4:$C$2000="Jonas")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
         <v/>
       </c>
-      <c r="E115" s="32">
+      <c r="E115" s="33">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=4)*('Lead-Tracking 2026'!$C$4:$C$2000="Angie")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
         <v/>
       </c>
-      <c r="F115" s="32">
+      <c r="F115" s="33">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=4)*('Lead-Tracking 2026'!$C$4:$C$2000="Norbert")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
         <v/>
       </c>
-      <c r="G115" s="32">
+      <c r="G115" s="33">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=4)*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
         <v/>
       </c>
-      <c r="H115" s="32">
+      <c r="H115" s="33">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=4)*('Lead-Tracking 2026'!$C$4:$C$2000="Daniel")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
         <v/>
       </c>
-      <c r="I115" s="32">
+      <c r="I115" s="33">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=4)*('Lead-Tracking 2026'!$C$4:$C$2000="Jonas")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
         <v/>
       </c>
-      <c r="J115" s="32">
+      <c r="J115" s="33">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=4)*('Lead-Tracking 2026'!$C$4:$C$2000="Angie")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
         <v/>
       </c>
-      <c r="K115" s="32">
+      <c r="K115" s="33">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=4)*('Lead-Tracking 2026'!$C$4:$C$2000="Norbert")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
         <v/>
       </c>
-      <c r="L115" s="32">
+      <c r="L115" s="33">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=4)*('Lead-Tracking 2026'!$A$4:$A$2000&lt;&gt;""))</f>
         <v/>
       </c>
-      <c r="M115" s="32">
+      <c r="M115" s="33">
         <f>M114+B115</f>
         <v/>
       </c>
     </row>
     <row r="116" ht="18" customHeight="1">
-      <c r="A116" s="29" t="inlineStr">
+      <c r="A116" s="30" t="inlineStr">
         <is>
           <t>Mai</t>
         </is>
       </c>
-      <c r="B116" s="30">
+      <c r="B116" s="31">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=5)*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
         <v/>
       </c>
-      <c r="C116" s="30">
+      <c r="C116" s="31">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=5)*('Lead-Tracking 2026'!$C$4:$C$2000="Daniel")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
         <v/>
       </c>
-      <c r="D116" s="30">
+      <c r="D116" s="31">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=5)*('Lead-Tracking 2026'!$C$4:$C$2000="Jonas")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
         <v/>
       </c>
-      <c r="E116" s="30">
+      <c r="E116" s="31">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=5)*('Lead-Tracking 2026'!$C$4:$C$2000="Angie")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
         <v/>
       </c>
-      <c r="F116" s="30">
+      <c r="F116" s="31">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=5)*('Lead-Tracking 2026'!$C$4:$C$2000="Norbert")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
         <v/>
       </c>
-      <c r="G116" s="30">
+      <c r="G116" s="31">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=5)*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
         <v/>
       </c>
-      <c r="H116" s="30">
+      <c r="H116" s="31">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=5)*('Lead-Tracking 2026'!$C$4:$C$2000="Daniel")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
         <v/>
       </c>
-      <c r="I116" s="30">
+      <c r="I116" s="31">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=5)*('Lead-Tracking 2026'!$C$4:$C$2000="Jonas")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
         <v/>
       </c>
-      <c r="J116" s="30">
+      <c r="J116" s="31">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=5)*('Lead-Tracking 2026'!$C$4:$C$2000="Angie")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
         <v/>
       </c>
-      <c r="K116" s="30">
+      <c r="K116" s="31">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=5)*('Lead-Tracking 2026'!$C$4:$C$2000="Norbert")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
         <v/>
       </c>
-      <c r="L116" s="30">
+      <c r="L116" s="31">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=5)*('Lead-Tracking 2026'!$A$4:$A$2000&lt;&gt;""))</f>
         <v/>
       </c>
-      <c r="M116" s="30">
+      <c r="M116" s="31">
         <f>M115+B116</f>
         <v/>
       </c>
     </row>
     <row r="117" ht="18" customHeight="1">
-      <c r="A117" s="31" t="inlineStr">
+      <c r="A117" s="32" t="inlineStr">
         <is>
           <t>Juni</t>
         </is>
       </c>
-      <c r="B117" s="32">
+      <c r="B117" s="33">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=6)*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
         <v/>
       </c>
-      <c r="C117" s="32">
+      <c r="C117" s="33">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=6)*('Lead-Tracking 2026'!$C$4:$C$2000="Daniel")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
         <v/>
       </c>
-      <c r="D117" s="32">
+      <c r="D117" s="33">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=6)*('Lead-Tracking 2026'!$C$4:$C$2000="Jonas")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
         <v/>
       </c>
-      <c r="E117" s="32">
+      <c r="E117" s="33">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=6)*('Lead-Tracking 2026'!$C$4:$C$2000="Angie")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
         <v/>
       </c>
-      <c r="F117" s="32">
+      <c r="F117" s="33">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=6)*('Lead-Tracking 2026'!$C$4:$C$2000="Norbert")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
         <v/>
       </c>
-      <c r="G117" s="32">
+      <c r="G117" s="33">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=6)*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
         <v/>
       </c>
-      <c r="H117" s="32">
+      <c r="H117" s="33">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=6)*('Lead-Tracking 2026'!$C$4:$C$2000="Daniel")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
         <v/>
       </c>
-      <c r="I117" s="32">
+      <c r="I117" s="33">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=6)*('Lead-Tracking 2026'!$C$4:$C$2000="Jonas")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
         <v/>
       </c>
-      <c r="J117" s="32">
+      <c r="J117" s="33">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=6)*('Lead-Tracking 2026'!$C$4:$C$2000="Angie")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
         <v/>
       </c>
-      <c r="K117" s="32">
+      <c r="K117" s="33">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=6)*('Lead-Tracking 2026'!$C$4:$C$2000="Norbert")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
         <v/>
       </c>
-      <c r="L117" s="32">
+      <c r="L117" s="33">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=6)*('Lead-Tracking 2026'!$A$4:$A$2000&lt;&gt;""))</f>
         <v/>
       </c>
-      <c r="M117" s="32">
+      <c r="M117" s="33">
         <f>M116+B117</f>
         <v/>
       </c>
     </row>
     <row r="118" ht="18" customHeight="1">
-      <c r="A118" s="29" t="inlineStr">
+      <c r="A118" s="30" t="inlineStr">
         <is>
           <t>Juli</t>
         </is>
       </c>
-      <c r="B118" s="30">
+      <c r="B118" s="31">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=7)*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
         <v/>
       </c>
-      <c r="C118" s="30">
+      <c r="C118" s="31">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=7)*('Lead-Tracking 2026'!$C$4:$C$2000="Daniel")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
         <v/>
       </c>
-      <c r="D118" s="30">
+      <c r="D118" s="31">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=7)*('Lead-Tracking 2026'!$C$4:$C$2000="Jonas")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
         <v/>
       </c>
-      <c r="E118" s="30">
+      <c r="E118" s="31">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=7)*('Lead-Tracking 2026'!$C$4:$C$2000="Angie")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
         <v/>
       </c>
-      <c r="F118" s="30">
+      <c r="F118" s="31">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=7)*('Lead-Tracking 2026'!$C$4:$C$2000="Norbert")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
         <v/>
       </c>
-      <c r="G118" s="30">
+      <c r="G118" s="31">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=7)*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
         <v/>
       </c>
-      <c r="H118" s="30">
+      <c r="H118" s="31">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=7)*('Lead-Tracking 2026'!$C$4:$C$2000="Daniel")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
         <v/>
       </c>
-      <c r="I118" s="30">
+      <c r="I118" s="31">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=7)*('Lead-Tracking 2026'!$C$4:$C$2000="Jonas")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
         <v/>
       </c>
-      <c r="J118" s="30">
+      <c r="J118" s="31">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=7)*('Lead-Tracking 2026'!$C$4:$C$2000="Angie")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
         <v/>
       </c>
-      <c r="K118" s="30">
+      <c r="K118" s="31">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=7)*('Lead-Tracking 2026'!$C$4:$C$2000="Norbert")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
         <v/>
       </c>
-      <c r="L118" s="30">
+      <c r="L118" s="31">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=7)*('Lead-Tracking 2026'!$A$4:$A$2000&lt;&gt;""))</f>
         <v/>
       </c>
-      <c r="M118" s="30">
+      <c r="M118" s="31">
         <f>M117+B118</f>
         <v/>
       </c>
     </row>
     <row r="119" ht="18" customHeight="1">
-      <c r="A119" s="31" t="inlineStr">
+      <c r="A119" s="32" t="inlineStr">
         <is>
           <t>August</t>
         </is>
       </c>
-      <c r="B119" s="32">
+      <c r="B119" s="33">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=8)*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
         <v/>
       </c>
-      <c r="C119" s="32">
+      <c r="C119" s="33">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=8)*('Lead-Tracking 2026'!$C$4:$C$2000="Daniel")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
         <v/>
       </c>
-      <c r="D119" s="32">
+      <c r="D119" s="33">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=8)*('Lead-Tracking 2026'!$C$4:$C$2000="Jonas")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
         <v/>
       </c>
-      <c r="E119" s="32">
+      <c r="E119" s="33">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=8)*('Lead-Tracking 2026'!$C$4:$C$2000="Angie")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
         <v/>
       </c>
-      <c r="F119" s="32">
+      <c r="F119" s="33">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=8)*('Lead-Tracking 2026'!$C$4:$C$2000="Norbert")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
         <v/>
       </c>
-      <c r="G119" s="32">
+      <c r="G119" s="33">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=8)*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
         <v/>
       </c>
-      <c r="H119" s="32">
+      <c r="H119" s="33">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=8)*('Lead-Tracking 2026'!$C$4:$C$2000="Daniel")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
         <v/>
       </c>
-      <c r="I119" s="32">
+      <c r="I119" s="33">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=8)*('Lead-Tracking 2026'!$C$4:$C$2000="Jonas")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
         <v/>
       </c>
-      <c r="J119" s="32">
+      <c r="J119" s="33">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=8)*('Lead-Tracking 2026'!$C$4:$C$2000="Angie")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
         <v/>
       </c>
-      <c r="K119" s="32">
+      <c r="K119" s="33">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=8)*('Lead-Tracking 2026'!$C$4:$C$2000="Norbert")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
         <v/>
       </c>
-      <c r="L119" s="32">
+      <c r="L119" s="33">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=8)*('Lead-Tracking 2026'!$A$4:$A$2000&lt;&gt;""))</f>
         <v/>
       </c>
-      <c r="M119" s="32">
+      <c r="M119" s="33">
         <f>M118+B119</f>
         <v/>
       </c>
     </row>
     <row r="120" ht="18" customHeight="1">
-      <c r="A120" s="29" t="inlineStr">
+      <c r="A120" s="30" t="inlineStr">
         <is>
           <t>September</t>
         </is>
       </c>
-      <c r="B120" s="30">
+      <c r="B120" s="31">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=9)*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
         <v/>
       </c>
-      <c r="C120" s="30">
+      <c r="C120" s="31">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=9)*('Lead-Tracking 2026'!$C$4:$C$2000="Daniel")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
         <v/>
       </c>
-      <c r="D120" s="30">
+      <c r="D120" s="31">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=9)*('Lead-Tracking 2026'!$C$4:$C$2000="Jonas")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
         <v/>
       </c>
-      <c r="E120" s="30">
+      <c r="E120" s="31">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=9)*('Lead-Tracking 2026'!$C$4:$C$2000="Angie")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
         <v/>
       </c>
-      <c r="F120" s="30">
+      <c r="F120" s="31">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=9)*('Lead-Tracking 2026'!$C$4:$C$2000="Norbert")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
         <v/>
       </c>
-      <c r="G120" s="30">
+      <c r="G120" s="31">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=9)*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
         <v/>
       </c>
-      <c r="H120" s="30">
+      <c r="H120" s="31">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=9)*('Lead-Tracking 2026'!$C$4:$C$2000="Daniel")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
         <v/>
       </c>
-      <c r="I120" s="30">
+      <c r="I120" s="31">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=9)*('Lead-Tracking 2026'!$C$4:$C$2000="Jonas")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
         <v/>
       </c>
-      <c r="J120" s="30">
+      <c r="J120" s="31">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=9)*('Lead-Tracking 2026'!$C$4:$C$2000="Angie")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
         <v/>
       </c>
-      <c r="K120" s="30">
+      <c r="K120" s="31">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=9)*('Lead-Tracking 2026'!$C$4:$C$2000="Norbert")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
         <v/>
       </c>
-      <c r="L120" s="30">
+      <c r="L120" s="31">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=9)*('Lead-Tracking 2026'!$A$4:$A$2000&lt;&gt;""))</f>
         <v/>
       </c>
-      <c r="M120" s="30">
+      <c r="M120" s="31">
         <f>M119+B120</f>
         <v/>
       </c>
     </row>
     <row r="121" ht="18" customHeight="1">
-      <c r="A121" s="31" t="inlineStr">
+      <c r="A121" s="32" t="inlineStr">
         <is>
           <t>Oktober</t>
         </is>
       </c>
-      <c r="B121" s="32">
+      <c r="B121" s="33">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=10)*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
         <v/>
       </c>
-      <c r="C121" s="32">
+      <c r="C121" s="33">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=10)*('Lead-Tracking 2026'!$C$4:$C$2000="Daniel")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
         <v/>
       </c>
-      <c r="D121" s="32">
+      <c r="D121" s="33">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=10)*('Lead-Tracking 2026'!$C$4:$C$2000="Jonas")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
         <v/>
       </c>
-      <c r="E121" s="32">
+      <c r="E121" s="33">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=10)*('Lead-Tracking 2026'!$C$4:$C$2000="Angie")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
         <v/>
       </c>
-      <c r="F121" s="32">
+      <c r="F121" s="33">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=10)*('Lead-Tracking 2026'!$C$4:$C$2000="Norbert")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
         <v/>
       </c>
-      <c r="G121" s="32">
+      <c r="G121" s="33">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=10)*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
         <v/>
       </c>
-      <c r="H121" s="32">
+      <c r="H121" s="33">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=10)*('Lead-Tracking 2026'!$C$4:$C$2000="Daniel")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
         <v/>
       </c>
-      <c r="I121" s="32">
+      <c r="I121" s="33">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=10)*('Lead-Tracking 2026'!$C$4:$C$2000="Jonas")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
         <v/>
       </c>
-      <c r="J121" s="32">
+      <c r="J121" s="33">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=10)*('Lead-Tracking 2026'!$C$4:$C$2000="Angie")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
         <v/>
       </c>
-      <c r="K121" s="32">
+      <c r="K121" s="33">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=10)*('Lead-Tracking 2026'!$C$4:$C$2000="Norbert")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
         <v/>
       </c>
-      <c r="L121" s="32">
+      <c r="L121" s="33">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=10)*('Lead-Tracking 2026'!$A$4:$A$2000&lt;&gt;""))</f>
         <v/>
       </c>
-      <c r="M121" s="32">
+      <c r="M121" s="33">
         <f>M120+B121</f>
         <v/>
       </c>
     </row>
     <row r="122" ht="18" customHeight="1">
-      <c r="A122" s="29" t="inlineStr">
+      <c r="A122" s="30" t="inlineStr">
         <is>
           <t>November</t>
         </is>
       </c>
-      <c r="B122" s="30">
+      <c r="B122" s="31">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=11)*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
         <v/>
       </c>
-      <c r="C122" s="30">
+      <c r="C122" s="31">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=11)*('Lead-Tracking 2026'!$C$4:$C$2000="Daniel")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
         <v/>
       </c>
-      <c r="D122" s="30">
+      <c r="D122" s="31">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=11)*('Lead-Tracking 2026'!$C$4:$C$2000="Jonas")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
         <v/>
       </c>
-      <c r="E122" s="30">
+      <c r="E122" s="31">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=11)*('Lead-Tracking 2026'!$C$4:$C$2000="Angie")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
         <v/>
       </c>
-      <c r="F122" s="30">
+      <c r="F122" s="31">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=11)*('Lead-Tracking 2026'!$C$4:$C$2000="Norbert")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
         <v/>
       </c>
-      <c r="G122" s="30">
+      <c r="G122" s="31">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=11)*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
         <v/>
       </c>
-      <c r="H122" s="30">
+      <c r="H122" s="31">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=11)*('Lead-Tracking 2026'!$C$4:$C$2000="Daniel")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
         <v/>
       </c>
-      <c r="I122" s="30">
+      <c r="I122" s="31">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=11)*('Lead-Tracking 2026'!$C$4:$C$2000="Jonas")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
         <v/>
       </c>
-      <c r="J122" s="30">
+      <c r="J122" s="31">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=11)*('Lead-Tracking 2026'!$C$4:$C$2000="Angie")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
         <v/>
       </c>
-      <c r="K122" s="30">
+      <c r="K122" s="31">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=11)*('Lead-Tracking 2026'!$C$4:$C$2000="Norbert")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
         <v/>
       </c>
-      <c r="L122" s="30">
+      <c r="L122" s="31">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=11)*('Lead-Tracking 2026'!$A$4:$A$2000&lt;&gt;""))</f>
         <v/>
       </c>
-      <c r="M122" s="30">
+      <c r="M122" s="31">
         <f>M121+B122</f>
         <v/>
       </c>
     </row>
     <row r="123" ht="18" customHeight="1">
-      <c r="A123" s="31" t="inlineStr">
+      <c r="A123" s="32" t="inlineStr">
         <is>
           <t>Dezember</t>
         </is>
       </c>
-      <c r="B123" s="32">
+      <c r="B123" s="33">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=12)*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
         <v/>
       </c>
-      <c r="C123" s="32">
+      <c r="C123" s="33">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=12)*('Lead-Tracking 2026'!$C$4:$C$2000="Daniel")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
         <v/>
       </c>
-      <c r="D123" s="32">
+      <c r="D123" s="33">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=12)*('Lead-Tracking 2026'!$C$4:$C$2000="Jonas")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
         <v/>
       </c>
-      <c r="E123" s="32">
+      <c r="E123" s="33">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=12)*('Lead-Tracking 2026'!$C$4:$C$2000="Angie")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
         <v/>
       </c>
-      <c r="F123" s="32">
+      <c r="F123" s="33">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=12)*('Lead-Tracking 2026'!$C$4:$C$2000="Norbert")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja")*('Lead-Tracking 2026'!$P$4:$P$2000))</f>
         <v/>
       </c>
-      <c r="G123" s="32">
+      <c r="G123" s="33">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=12)*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
         <v/>
       </c>
-      <c r="H123" s="32">
+      <c r="H123" s="33">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=12)*('Lead-Tracking 2026'!$C$4:$C$2000="Daniel")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
         <v/>
       </c>
-      <c r="I123" s="32">
+      <c r="I123" s="33">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=12)*('Lead-Tracking 2026'!$C$4:$C$2000="Jonas")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
         <v/>
       </c>
-      <c r="J123" s="32">
+      <c r="J123" s="33">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=12)*('Lead-Tracking 2026'!$C$4:$C$2000="Angie")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
         <v/>
       </c>
-      <c r="K123" s="32">
+      <c r="K123" s="33">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=12)*('Lead-Tracking 2026'!$C$4:$C$2000="Norbert")*('Lead-Tracking 2026'!$Q$4:$Q$2000="Ja"))</f>
         <v/>
       </c>
-      <c r="L123" s="32">
+      <c r="L123" s="33">
         <f>SUMPRODUCT((YEAR('Lead-Tracking 2026'!$B$4:$B$2000)=2026)*(MONTH('Lead-Tracking 2026'!$B$4:$B$2000)=12)*('Lead-Tracking 2026'!$A$4:$A$2000&lt;&gt;""))</f>
         <v/>
       </c>
-      <c r="M123" s="32">
+      <c r="M123" s="33">
         <f>M122+B123</f>
         <v/>
       </c>
@@ -7962,7 +7348,6 @@
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -8002,17 +7387,17 @@
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="33" t="inlineStr">
+      <c r="A5" s="34" t="inlineStr">
         <is>
           <t>Kuerzel</t>
         </is>
       </c>
-      <c r="B5" s="33" t="inlineStr">
+      <c r="B5" s="34" t="inlineStr">
         <is>
           <t>Beschreibung</t>
         </is>
       </c>
-      <c r="C5" s="33" t="inlineStr">
+      <c r="C5" s="34" t="inlineStr">
         <is>
           <t>Strategie</t>
         </is>
@@ -8196,17 +7581,17 @@
       </c>
     </row>
     <row r="18" ht="20" customHeight="1">
-      <c r="A18" s="33" t="inlineStr">
+      <c r="A18" s="34" t="inlineStr">
         <is>
           <t>Code</t>
         </is>
       </c>
-      <c r="B18" s="33" t="inlineStr">
+      <c r="B18" s="34" t="inlineStr">
         <is>
           <t>Kunden-Formulierung / Bedeutung</t>
         </is>
       </c>
-      <c r="C18" s="33" t="inlineStr">
+      <c r="C18" s="34" t="inlineStr">
         <is>
           <t>Naechster Schritt</t>
         </is>
@@ -8390,48 +7775,48 @@
       </c>
     </row>
     <row r="31" ht="18" customHeight="1">
-      <c r="A31" s="34" t="inlineStr">
+      <c r="A31" s="35" t="inlineStr">
         <is>
           <t>ok</t>
         </is>
       </c>
-      <c r="B31" s="35" t="inlineStr">
+      <c r="B31" s="36" t="inlineStr">
         <is>
           <t>Check-Datum liegt in &gt; 2 Tagen – alles im Plan</t>
         </is>
       </c>
     </row>
     <row r="32" ht="18" customHeight="1">
-      <c r="A32" s="36" t="inlineStr">
+      <c r="A32" s="37" t="inlineStr">
         <is>
           <t>~</t>
         </is>
       </c>
-      <c r="B32" s="37" t="inlineStr">
+      <c r="B32" s="38" t="inlineStr">
         <is>
           <t>Check-Datum heute oder morgen – sofort handeln</t>
         </is>
       </c>
     </row>
     <row r="33" ht="18" customHeight="1">
-      <c r="A33" s="38" t="inlineStr">
+      <c r="A33" s="39" t="inlineStr">
         <is>
           <t>!</t>
         </is>
       </c>
-      <c r="B33" s="39" t="inlineStr">
+      <c r="B33" s="40" t="inlineStr">
         <is>
           <t>Check-Datum ueberschritten – dringend nachfassen!</t>
         </is>
       </c>
     </row>
     <row r="34" ht="18" customHeight="1">
-      <c r="A34" s="40" t="inlineStr">
+      <c r="A34" s="41" t="inlineStr">
         <is>
           <t>o</t>
         </is>
       </c>
-      <c r="B34" s="41" t="inlineStr">
+      <c r="B34" s="42" t="inlineStr">
         <is>
           <t>Abgeschlossen / Verloren / Wartet – kein Follow-up</t>
         </is>
@@ -8445,72 +7830,72 @@
       </c>
     </row>
     <row r="37" ht="18" customHeight="1">
-      <c r="A37" s="42" t="inlineStr">
+      <c r="A37" s="43" t="inlineStr">
         <is>
           <t>Kauf abgeschlossen</t>
         </is>
       </c>
-      <c r="B37" s="35" t="inlineStr">
+      <c r="B37" s="36" t="inlineStr">
         <is>
           <t>Abgeschlossen, kein Follow-up</t>
         </is>
       </c>
     </row>
     <row r="38" ht="18" customHeight="1">
-      <c r="A38" s="43" t="inlineStr">
+      <c r="A38" s="44" t="inlineStr">
         <is>
           <t>Heimcheck angelegt</t>
         </is>
       </c>
-      <c r="B38" s="44" t="inlineStr">
+      <c r="B38" s="45" t="inlineStr">
         <is>
           <t>Naechster Schritt: Check-Anruf</t>
         </is>
       </c>
     </row>
     <row r="39" ht="18" customHeight="1">
-      <c r="A39" s="45" t="inlineStr">
+      <c r="A39" s="46" t="inlineStr">
         <is>
           <t>Entscheidungscheck geplant</t>
         </is>
       </c>
-      <c r="B39" s="37" t="inlineStr">
+      <c r="B39" s="38" t="inlineStr">
         <is>
           <t>Kurz vor Abschluss – nachfassen</t>
         </is>
       </c>
     </row>
     <row r="40" ht="18" customHeight="1">
-      <c r="A40" s="46" t="inlineStr">
+      <c r="A40" s="47" t="inlineStr">
         <is>
           <t>Angebot konkret</t>
         </is>
       </c>
-      <c r="B40" s="47" t="inlineStr">
+      <c r="B40" s="48" t="inlineStr">
         <is>
           <t>Angebot liegt vor</t>
         </is>
       </c>
     </row>
     <row r="41" ht="18" customHeight="1">
-      <c r="A41" s="48" t="inlineStr">
+      <c r="A41" s="49" t="inlineStr">
         <is>
           <t>Verloren</t>
         </is>
       </c>
-      <c r="B41" s="39" t="inlineStr">
+      <c r="B41" s="40" t="inlineStr">
         <is>
           <t>Lead verloren – Verlustgrund eintragen</t>
         </is>
       </c>
     </row>
     <row r="42" ht="18" customHeight="1">
-      <c r="A42" s="49" t="inlineStr">
+      <c r="A42" s="50" t="inlineStr">
         <is>
           <t>Warten auf Raum</t>
         </is>
       </c>
-      <c r="B42" s="41" t="inlineStr">
+      <c r="B42" s="42" t="inlineStr">
         <is>
           <t>Wiedervorlage in Monaten</t>
         </is>
@@ -8524,36 +7909,36 @@
       </c>
     </row>
     <row r="45" ht="18" customHeight="1">
-      <c r="A45" s="50" t="inlineStr">
+      <c r="A45" s="51" t="inlineStr">
         <is>
           <t>Ja</t>
         </is>
       </c>
-      <c r="B45" s="35" t="inlineStr">
+      <c r="B45" s="36" t="inlineStr">
         <is>
           <t>Verkauf abgeschlossen</t>
         </is>
       </c>
     </row>
     <row r="46" ht="18" customHeight="1">
-      <c r="A46" s="51" t="inlineStr">
+      <c r="A46" s="52" t="inlineStr">
         <is>
           <t>Offen</t>
         </is>
       </c>
-      <c r="B46" s="37" t="inlineStr">
+      <c r="B46" s="38" t="inlineStr">
         <is>
           <t>Lead laeuft noch – dranbleiben</t>
         </is>
       </c>
     </row>
     <row r="47" ht="18" customHeight="1">
-      <c r="A47" s="52" t="inlineStr">
+      <c r="A47" s="53" t="inlineStr">
         <is>
           <t>Nein</t>
         </is>
       </c>
-      <c r="B47" s="39" t="inlineStr">
+      <c r="B47" s="40" t="inlineStr">
         <is>
           <t>Lead verloren – Verlustgrund eintragen</t>
         </is>
@@ -8567,36 +7952,36 @@
       </c>
     </row>
     <row r="51" ht="18" customHeight="1">
-      <c r="A51" s="50" t="inlineStr">
+      <c r="A51" s="51" t="inlineStr">
         <is>
           <t>&gt; 60 %</t>
         </is>
       </c>
-      <c r="B51" s="35" t="inlineStr">
+      <c r="B51" s="36" t="inlineStr">
         <is>
           <t>Top – Ziel uebertroffen</t>
         </is>
       </c>
     </row>
     <row r="52" ht="18" customHeight="1">
-      <c r="A52" s="51" t="inlineStr">
+      <c r="A52" s="52" t="inlineStr">
         <is>
           <t>40 – 60 %</t>
         </is>
       </c>
-      <c r="B52" s="37" t="inlineStr">
+      <c r="B52" s="38" t="inlineStr">
         <is>
           <t>Solide – im Zielkorridor</t>
         </is>
       </c>
     </row>
     <row r="53" ht="18" customHeight="1">
-      <c r="A53" s="52" t="inlineStr">
+      <c r="A53" s="53" t="inlineStr">
         <is>
           <t>&lt; 40 %</t>
         </is>
       </c>
-      <c r="B53" s="39" t="inlineStr">
+      <c r="B53" s="40" t="inlineStr">
         <is>
           <t>Unter Soll – Prozess pruefen</t>
         </is>

</xml_diff>